<commit_message>
Add "Website by BISCS India" credit to the footer
Links to https://www.biscsindia.com from the footer's bottom bar on every
page. Text and link are editable in the Google Sheet (Company tab); empty
text hides the credit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_019FQMsi9UwAgehJoy2UKmFf
</commit_message>
<xml_diff>
--- a/google-sheets/Kunnect-Website-Content.xlsx
+++ b/google-sheets/Kunnect-Website-Content.xlsx
@@ -309,7 +309,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5371" uniqueCount="592">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5379" uniqueCount="599">
   <si>
     <t>Kunnect website content</t>
   </si>
@@ -522,6 +522,27 @@
   </si>
   <si>
     <t>Strategic digital marketing and custom software for small and medium-scale businesses.</t>
+  </si>
+  <si>
+    <t>footer.credit_text</t>
+  </si>
+  <si>
+    <t>Website credit text</t>
+  </si>
+  <si>
+    <t>Website by BISCS India</t>
+  </si>
+  <si>
+    <t>Shown at the bottom of every page. Leave empty to hide.</t>
+  </si>
+  <si>
+    <t>footer.credit_link</t>
+  </si>
+  <si>
+    <t>Website credit link</t>
+  </si>
+  <si>
+    <t>https://www.biscsindia.com</t>
   </si>
   <si>
     <t>launch.hide_placeholders</t>
@@ -2797,7 +2818,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>377</v>
+        <v>384</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -2820,96 +2841,96 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>379</v>
+        <v>386</v>
       </c>
       <c r="D2" s="7" t="s">
         <v>29</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>380</v>
+        <v>387</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>382</v>
+        <v>389</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>383</v>
+        <v>390</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>384</v>
+        <v>391</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>385</v>
+        <v>392</v>
       </c>
       <c r="K2" s="7" t="s">
-        <v>386</v>
+        <v>393</v>
       </c>
       <c r="L2" s="7" t="s">
-        <v>387</v>
+        <v>394</v>
       </c>
       <c r="M2" s="7" t="s">
-        <v>388</v>
+        <v>395</v>
       </c>
       <c r="N2" s="7" t="s">
-        <v>389</v>
+        <v>396</v>
       </c>
       <c r="O2" s="7" t="s">
-        <v>390</v>
+        <v>397</v>
       </c>
       <c r="P2" s="7" t="s">
-        <v>391</v>
+        <v>398</v>
       </c>
       <c r="Q2" s="7" t="s">
-        <v>392</v>
+        <v>399</v>
       </c>
       <c r="R2" s="7" t="s">
-        <v>393</v>
+        <v>400</v>
       </c>
       <c r="S2" s="7" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>394</v>
+        <v>401</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>395</v>
+        <v>402</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>396</v>
+        <v>403</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>398</v>
+        <v>405</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>399</v>
+        <v>406</v>
       </c>
       <c r="H3" s="10" t="s">
-        <v>400</v>
+        <v>407</v>
       </c>
       <c r="I3" s="10" t="s">
-        <v>401</v>
+        <v>408</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>402</v>
+        <v>409</v>
       </c>
       <c r="K3" s="10" t="s">
-        <v>403</v>
+        <v>410</v>
       </c>
       <c r="L3" s="10" t="s">
         <v>2</v>
@@ -2927,10 +2948,10 @@
         <v>2</v>
       </c>
       <c r="Q3" s="10" t="s">
-        <v>404</v>
+        <v>411</v>
       </c>
       <c r="R3" s="10" t="s">
-        <v>405</v>
+        <v>412</v>
       </c>
       <c r="S3" s="10" t="s">
         <v>2</v>
@@ -2938,37 +2959,37 @@
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>406</v>
+        <v>413</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>407</v>
+        <v>414</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>408</v>
+        <v>415</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>409</v>
+        <v>416</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>410</v>
+        <v>417</v>
       </c>
       <c r="H4" s="10" t="s">
-        <v>411</v>
+        <v>418</v>
       </c>
       <c r="I4" s="10" t="s">
-        <v>412</v>
+        <v>419</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>413</v>
+        <v>420</v>
       </c>
       <c r="K4" s="10" t="s">
-        <v>414</v>
+        <v>421</v>
       </c>
       <c r="L4" s="10" t="s">
         <v>2</v>
@@ -2986,10 +3007,10 @@
         <v>2</v>
       </c>
       <c r="Q4" s="10" t="s">
-        <v>415</v>
+        <v>422</v>
       </c>
       <c r="R4" s="10" t="s">
-        <v>416</v>
+        <v>423</v>
       </c>
       <c r="S4" s="10" t="s">
         <v>2</v>
@@ -2997,37 +3018,37 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>417</v>
+        <v>424</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>418</v>
+        <v>425</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>419</v>
+        <v>426</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>420</v>
+        <v>427</v>
       </c>
       <c r="H5" s="10" t="s">
-        <v>421</v>
+        <v>428</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>422</v>
+        <v>429</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>423</v>
+        <v>430</v>
       </c>
       <c r="K5" s="10" t="s">
-        <v>424</v>
+        <v>431</v>
       </c>
       <c r="L5" s="10" t="s">
         <v>2</v>
@@ -3045,10 +3066,10 @@
         <v>2</v>
       </c>
       <c r="Q5" s="10" t="s">
-        <v>425</v>
+        <v>432</v>
       </c>
       <c r="R5" s="10" t="s">
-        <v>426</v>
+        <v>433</v>
       </c>
       <c r="S5" s="10" t="s">
         <v>2</v>
@@ -3056,37 +3077,37 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>427</v>
+        <v>434</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>428</v>
+        <v>435</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>429</v>
+        <v>436</v>
       </c>
       <c r="E6" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>430</v>
+        <v>437</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>431</v>
+        <v>438</v>
       </c>
       <c r="H6" s="10" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="I6" s="10" t="s">
-        <v>433</v>
+        <v>440</v>
       </c>
       <c r="J6" s="10" t="s">
-        <v>434</v>
+        <v>441</v>
       </c>
       <c r="K6" s="10" t="s">
-        <v>435</v>
+        <v>442</v>
       </c>
       <c r="L6" s="10" t="s">
         <v>2</v>
@@ -3104,10 +3125,10 @@
         <v>2</v>
       </c>
       <c r="Q6" s="10" t="s">
-        <v>436</v>
+        <v>443</v>
       </c>
       <c r="R6" s="10" t="s">
-        <v>437</v>
+        <v>444</v>
       </c>
       <c r="S6" s="10" t="s">
         <v>2</v>
@@ -3115,37 +3136,37 @@
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>438</v>
+        <v>445</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>439</v>
+        <v>446</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>440</v>
+        <v>447</v>
       </c>
       <c r="E7" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>441</v>
+        <v>448</v>
       </c>
       <c r="G7" s="10" t="s">
-        <v>442</v>
+        <v>449</v>
       </c>
       <c r="H7" s="10" t="s">
-        <v>443</v>
+        <v>450</v>
       </c>
       <c r="I7" s="10" t="s">
-        <v>444</v>
+        <v>451</v>
       </c>
       <c r="J7" s="10" t="s">
-        <v>445</v>
+        <v>452</v>
       </c>
       <c r="K7" s="10" t="s">
-        <v>446</v>
+        <v>453</v>
       </c>
       <c r="L7" s="10" t="s">
         <v>2</v>
@@ -3163,10 +3184,10 @@
         <v>2</v>
       </c>
       <c r="Q7" s="10" t="s">
-        <v>447</v>
+        <v>454</v>
       </c>
       <c r="R7" s="10" t="s">
-        <v>448</v>
+        <v>455</v>
       </c>
       <c r="S7" s="10" t="s">
         <v>2</v>
@@ -3174,37 +3195,37 @@
     </row>
     <row r="8" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>449</v>
+        <v>456</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>450</v>
+        <v>457</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>451</v>
+        <v>458</v>
       </c>
       <c r="E8" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>452</v>
+        <v>459</v>
       </c>
       <c r="G8" s="10" t="s">
-        <v>453</v>
+        <v>460</v>
       </c>
       <c r="H8" s="10" t="s">
-        <v>454</v>
+        <v>461</v>
       </c>
       <c r="I8" s="10" t="s">
-        <v>455</v>
+        <v>462</v>
       </c>
       <c r="J8" s="10" t="s">
-        <v>456</v>
+        <v>463</v>
       </c>
       <c r="K8" s="10" t="s">
-        <v>457</v>
+        <v>464</v>
       </c>
       <c r="L8" s="10" t="s">
         <v>2</v>
@@ -3222,10 +3243,10 @@
         <v>2</v>
       </c>
       <c r="Q8" s="10" t="s">
-        <v>458</v>
+        <v>465</v>
       </c>
       <c r="R8" s="10" t="s">
-        <v>459</v>
+        <v>466</v>
       </c>
       <c r="S8" s="10" t="s">
         <v>2</v>
@@ -3233,37 +3254,37 @@
     </row>
     <row r="9" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>460</v>
+        <v>467</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>461</v>
+        <v>468</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>462</v>
+        <v>469</v>
       </c>
       <c r="E9" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>463</v>
+        <v>470</v>
       </c>
       <c r="G9" s="10" t="s">
-        <v>464</v>
+        <v>471</v>
       </c>
       <c r="H9" s="10" t="s">
-        <v>465</v>
+        <v>472</v>
       </c>
       <c r="I9" s="10" t="s">
-        <v>466</v>
+        <v>473</v>
       </c>
       <c r="J9" s="10" t="s">
-        <v>467</v>
+        <v>474</v>
       </c>
       <c r="K9" s="10" t="s">
-        <v>468</v>
+        <v>475</v>
       </c>
       <c r="L9" s="10" t="s">
         <v>2</v>
@@ -3281,10 +3302,10 @@
         <v>2</v>
       </c>
       <c r="Q9" s="10" t="s">
-        <v>469</v>
+        <v>476</v>
       </c>
       <c r="R9" s="10" t="s">
-        <v>470</v>
+        <v>477</v>
       </c>
       <c r="S9" s="10" t="s">
         <v>2</v>
@@ -3292,37 +3313,37 @@
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>471</v>
+        <v>478</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>472</v>
+        <v>479</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>473</v>
+        <v>480</v>
       </c>
       <c r="E10" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>474</v>
+        <v>481</v>
       </c>
       <c r="G10" s="10" t="s">
-        <v>475</v>
+        <v>482</v>
       </c>
       <c r="H10" s="10" t="s">
-        <v>476</v>
+        <v>483</v>
       </c>
       <c r="I10" s="10" t="s">
-        <v>477</v>
+        <v>484</v>
       </c>
       <c r="J10" s="10" t="s">
-        <v>478</v>
+        <v>485</v>
       </c>
       <c r="K10" s="10" t="s">
-        <v>479</v>
+        <v>486</v>
       </c>
       <c r="L10" s="10" t="s">
         <v>2</v>
@@ -3340,10 +3361,10 @@
         <v>2</v>
       </c>
       <c r="Q10" s="10" t="s">
-        <v>480</v>
+        <v>487</v>
       </c>
       <c r="R10" s="10" t="s">
-        <v>481</v>
+        <v>488</v>
       </c>
       <c r="S10" s="10" t="s">
         <v>2</v>
@@ -3351,37 +3372,37 @@
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A11" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>483</v>
+        <v>490</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>482</v>
+        <v>489</v>
       </c>
       <c r="E11" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F11" s="10" t="s">
-        <v>484</v>
+        <v>491</v>
       </c>
       <c r="G11" s="10" t="s">
-        <v>485</v>
+        <v>492</v>
       </c>
       <c r="H11" s="10" t="s">
-        <v>486</v>
+        <v>493</v>
       </c>
       <c r="I11" s="10" t="s">
-        <v>487</v>
+        <v>494</v>
       </c>
       <c r="J11" s="10" t="s">
-        <v>488</v>
+        <v>495</v>
       </c>
       <c r="K11" s="10" t="s">
-        <v>489</v>
+        <v>496</v>
       </c>
       <c r="L11" s="10" t="s">
         <v>2</v>
@@ -3399,10 +3420,10 @@
         <v>2</v>
       </c>
       <c r="Q11" s="10" t="s">
-        <v>490</v>
+        <v>497</v>
       </c>
       <c r="R11" s="10" t="s">
-        <v>491</v>
+        <v>498</v>
       </c>
       <c r="S11" s="10" t="s">
         <v>2</v>
@@ -3410,37 +3431,37 @@
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A12" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B12" s="10" t="s">
-        <v>492</v>
+        <v>499</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>493</v>
+        <v>500</v>
       </c>
       <c r="D12" s="10" t="s">
-        <v>494</v>
+        <v>501</v>
       </c>
       <c r="E12" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F12" s="10" t="s">
-        <v>495</v>
+        <v>502</v>
       </c>
       <c r="G12" s="10" t="s">
-        <v>496</v>
+        <v>503</v>
       </c>
       <c r="H12" s="10" t="s">
-        <v>497</v>
+        <v>504</v>
       </c>
       <c r="I12" s="10" t="s">
-        <v>498</v>
+        <v>505</v>
       </c>
       <c r="J12" s="10" t="s">
-        <v>499</v>
+        <v>506</v>
       </c>
       <c r="K12" s="10" t="s">
-        <v>500</v>
+        <v>507</v>
       </c>
       <c r="L12" s="10" t="s">
         <v>2</v>
@@ -3458,10 +3479,10 @@
         <v>2</v>
       </c>
       <c r="Q12" s="10" t="s">
-        <v>501</v>
+        <v>508</v>
       </c>
       <c r="R12" s="10" t="s">
-        <v>502</v>
+        <v>509</v>
       </c>
       <c r="S12" s="10" t="s">
         <v>2</v>
@@ -3469,37 +3490,37 @@
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A13" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B13" s="10" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>503</v>
+        <v>510</v>
       </c>
       <c r="D13" s="10" t="s">
-        <v>504</v>
+        <v>511</v>
       </c>
       <c r="E13" s="10" t="s">
-        <v>397</v>
+        <v>404</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>505</v>
+        <v>512</v>
       </c>
       <c r="G13" s="10" t="s">
-        <v>506</v>
+        <v>513</v>
       </c>
       <c r="H13" s="10" t="s">
-        <v>507</v>
+        <v>514</v>
       </c>
       <c r="I13" s="10" t="s">
-        <v>508</v>
+        <v>515</v>
       </c>
       <c r="J13" s="10" t="s">
-        <v>509</v>
+        <v>516</v>
       </c>
       <c r="K13" s="10" t="s">
-        <v>510</v>
+        <v>517</v>
       </c>
       <c r="L13" s="10" t="s">
         <v>2</v>
@@ -3517,10 +3538,10 @@
         <v>2</v>
       </c>
       <c r="Q13" s="10" t="s">
-        <v>511</v>
+        <v>518</v>
       </c>
       <c r="R13" s="10" t="s">
-        <v>512</v>
+        <v>519</v>
       </c>
       <c r="S13" s="10" t="s">
         <v>2</v>
@@ -3528,37 +3549,37 @@
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A14" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>513</v>
+        <v>520</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>514</v>
+        <v>521</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>515</v>
+        <v>522</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>517</v>
+        <v>524</v>
       </c>
       <c r="G14" s="10" t="s">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="H14" s="10" t="s">
-        <v>519</v>
+        <v>526</v>
       </c>
       <c r="I14" s="10" t="s">
-        <v>520</v>
+        <v>527</v>
       </c>
       <c r="J14" s="10" t="s">
-        <v>521</v>
+        <v>528</v>
       </c>
       <c r="K14" s="10" t="s">
-        <v>522</v>
+        <v>529</v>
       </c>
       <c r="L14" s="10" t="s">
         <v>2</v>
@@ -3576,10 +3597,10 @@
         <v>2</v>
       </c>
       <c r="Q14" s="10" t="s">
-        <v>523</v>
+        <v>530</v>
       </c>
       <c r="R14" s="10" t="s">
-        <v>524</v>
+        <v>531</v>
       </c>
       <c r="S14" s="10" t="s">
         <v>2</v>
@@ -3587,37 +3608,37 @@
     </row>
     <row r="15" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A15" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B15" s="10" t="s">
-        <v>525</v>
+        <v>532</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>526</v>
+        <v>533</v>
       </c>
       <c r="D15" s="10" t="s">
-        <v>527</v>
+        <v>534</v>
       </c>
       <c r="E15" s="10" t="s">
-        <v>516</v>
+        <v>523</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>528</v>
+        <v>535</v>
       </c>
       <c r="G15" s="10" t="s">
-        <v>529</v>
+        <v>536</v>
       </c>
       <c r="H15" s="10" t="s">
-        <v>530</v>
+        <v>537</v>
       </c>
       <c r="I15" s="10" t="s">
-        <v>531</v>
+        <v>538</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>532</v>
+        <v>539</v>
       </c>
       <c r="K15" s="10" t="s">
-        <v>533</v>
+        <v>540</v>
       </c>
       <c r="L15" s="10" t="s">
         <v>2</v>
@@ -3635,10 +3656,10 @@
         <v>2</v>
       </c>
       <c r="Q15" s="10" t="s">
-        <v>534</v>
+        <v>541</v>
       </c>
       <c r="R15" s="10" t="s">
-        <v>535</v>
+        <v>542</v>
       </c>
       <c r="S15" s="10" t="s">
         <v>2</v>
@@ -7225,53 +7246,53 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>536</v>
+        <v>543</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>538</v>
+        <v>545</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>539</v>
+        <v>546</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>540</v>
+        <v>547</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>541</v>
+        <v>548</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>542</v>
+        <v>549</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>543</v>
+        <v>550</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -7963,7 +7984,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>544</v>
+        <v>551</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -7972,70 +7993,70 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>545</v>
+        <v>552</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>546</v>
+        <v>553</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>549</v>
+        <v>556</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>550</v>
+        <v>557</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>548</v>
+        <v>555</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>551</v>
+        <v>558</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>73</v>
+        <v>80</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -9093,53 +9114,53 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>552</v>
+        <v>559</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>553</v>
+        <v>560</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>554</v>
+        <v>561</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>555</v>
+        <v>562</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>556</v>
+        <v>563</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>557</v>
+        <v>564</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>558</v>
+        <v>565</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -9831,64 +9852,64 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>559</v>
+        <v>566</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>560</v>
+        <v>567</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>561</v>
+        <v>568</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>562</v>
+        <v>569</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>563</v>
+        <v>570</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>564</v>
+        <v>571</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>565</v>
+        <v>572</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>566</v>
+        <v>573</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>567</v>
+        <v>574</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -10581,7 +10602,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>568</v>
+        <v>575</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -10590,70 +10611,70 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>569</v>
+        <v>576</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="E3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="E4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>570</v>
+        <v>577</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>571</v>
+        <v>578</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>572</v>
+        <v>579</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -11712,7 +11733,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>573</v>
+        <v>580</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -11721,19 +11742,19 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>574</v>
+        <v>581</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>547</v>
+        <v>554</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -12791,53 +12812,53 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>575</v>
+        <v>582</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>378</v>
+        <v>385</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>537</v>
+        <v>544</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>576</v>
+        <v>583</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>577</v>
+        <v>584</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>578</v>
+        <v>585</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>579</v>
+        <v>586</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>580</v>
+        <v>587</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>581</v>
+        <v>588</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
@@ -13528,7 +13549,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>582</v>
+        <v>589</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -13536,27 +13557,27 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>381</v>
+        <v>388</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>583</v>
+        <v>590</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>584</v>
+        <v>591</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>585</v>
+        <v>592</v>
       </c>
       <c r="D3" s="10" t="s">
         <v>2</v>
@@ -13564,13 +13585,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>586</v>
+        <v>593</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>587</v>
+        <v>594</v>
       </c>
       <c r="D4" s="10" t="s">
         <v>2</v>
@@ -13578,13 +13599,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>588</v>
+        <v>595</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>589</v>
+        <v>596</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>2</v>
@@ -13592,13 +13613,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>590</v>
+        <v>597</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>591</v>
+        <v>598</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>2</v>
@@ -14470,7 +14491,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:D20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="26" customWidth="1"/>
@@ -14725,12 +14746,40 @@
         <v>74</v>
       </c>
     </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A19" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="B19" s="9" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="10" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" s="11" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A20" s="8" t="s">
+        <v>78</v>
+      </c>
+      <c r="B20" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="10" t="s">
+        <v>80</v>
+      </c>
+      <c r="D20" s="11" t="s">
+        <v>81</v>
+      </c>
+    </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D1"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Yes or No" error="Please choose Yes or No." sqref="C18">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" errorTitle="Yes or No" error="Please choose Yes or No." sqref="C20">
       <formula1>"Yes,No"</formula1>
     </dataValidation>
   </dataValidations>
@@ -14752,7 +14801,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>75</v>
+        <v>82</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -14774,13 +14823,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>76</v>
+        <v>83</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>77</v>
+        <v>84</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>78</v>
+        <v>85</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>2</v>
@@ -14788,13 +14837,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>2</v>
@@ -14802,27 +14851,27 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>83</v>
+        <v>90</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>88</v>
+        <v>95</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>2</v>
@@ -14830,13 +14879,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>90</v>
+        <v>97</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>2</v>
@@ -14844,13 +14893,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>92</v>
+        <v>99</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>93</v>
+        <v>100</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>2</v>
@@ -14858,13 +14907,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>95</v>
+        <v>102</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>96</v>
+        <v>103</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>2</v>
@@ -14872,13 +14921,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>98</v>
+        <v>105</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>99</v>
+        <v>106</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>2</v>
@@ -14886,13 +14935,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>101</v>
+        <v>108</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>102</v>
+        <v>109</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>103</v>
+        <v>110</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>2</v>
@@ -14900,13 +14949,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>104</v>
+        <v>111</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>105</v>
+        <v>112</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>2</v>
@@ -14914,13 +14963,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>107</v>
+        <v>114</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>108</v>
+        <v>115</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>109</v>
+        <v>116</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>2</v>
@@ -14928,13 +14977,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>111</v>
+        <v>118</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>112</v>
+        <v>119</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>2</v>
@@ -14942,27 +14991,27 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>113</v>
+        <v>120</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>114</v>
+        <v>121</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="D15" s="11" t="s">
-        <v>116</v>
+        <v>123</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>117</v>
+        <v>124</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>118</v>
+        <v>125</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>119</v>
+        <v>126</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>2</v>
@@ -14970,13 +15019,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>120</v>
+        <v>127</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>121</v>
+        <v>128</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>122</v>
+        <v>129</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>2</v>
@@ -14984,13 +15033,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>124</v>
+        <v>131</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>125</v>
+        <v>132</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>2</v>
@@ -14998,13 +15047,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>126</v>
+        <v>133</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>127</v>
+        <v>134</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>128</v>
+        <v>135</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>2</v>
@@ -15012,10 +15061,10 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>129</v>
+        <v>136</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>130</v>
+        <v>137</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>36</v>
@@ -15026,13 +15075,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>131</v>
+        <v>138</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>132</v>
+        <v>139</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>133</v>
+        <v>140</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>2</v>
@@ -15040,13 +15089,13 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>134</v>
+        <v>141</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>135</v>
+        <v>142</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>136</v>
+        <v>143</v>
       </c>
       <c r="D22" s="11" t="s">
         <v>2</v>
@@ -15054,13 +15103,13 @@
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>137</v>
+        <v>144</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>138</v>
+        <v>145</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>139</v>
+        <v>146</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>2</v>
@@ -15068,13 +15117,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>140</v>
+        <v>147</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>141</v>
+        <v>148</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>142</v>
+        <v>149</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>2</v>
@@ -15082,13 +15131,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>143</v>
+        <v>150</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>145</v>
+        <v>152</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>2</v>
@@ -15096,13 +15145,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>146</v>
+        <v>153</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>147</v>
+        <v>154</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>148</v>
+        <v>155</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>2</v>
@@ -15110,13 +15159,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>149</v>
+        <v>156</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>2</v>
@@ -15124,13 +15173,13 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>152</v>
+        <v>159</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>153</v>
+        <v>160</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>154</v>
+        <v>161</v>
       </c>
       <c r="D28" s="11" t="s">
         <v>2</v>
@@ -15138,27 +15187,27 @@
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>155</v>
+        <v>162</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>156</v>
+        <v>163</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>157</v>
+        <v>164</v>
       </c>
       <c r="D29" s="11" t="s">
-        <v>158</v>
+        <v>165</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>160</v>
+        <v>167</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>161</v>
+        <v>168</v>
       </c>
       <c r="D30" s="11" t="s">
         <v>2</v>
@@ -15166,13 +15215,13 @@
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="8" t="s">
-        <v>162</v>
+        <v>169</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>163</v>
+        <v>170</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>164</v>
+        <v>171</v>
       </c>
       <c r="D31" s="11" t="s">
         <v>2</v>
@@ -15180,13 +15229,13 @@
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
-        <v>165</v>
+        <v>172</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>166</v>
+        <v>173</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>91</v>
+        <v>98</v>
       </c>
       <c r="D32" s="11" t="s">
         <v>2</v>
@@ -15194,13 +15243,13 @@
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
-        <v>167</v>
+        <v>174</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>168</v>
+        <v>175</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>94</v>
+        <v>101</v>
       </c>
       <c r="D33" s="11" t="s">
         <v>2</v>
@@ -15208,13 +15257,13 @@
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
-        <v>169</v>
+        <v>176</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>170</v>
+        <v>177</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>97</v>
+        <v>104</v>
       </c>
       <c r="D34" s="11" t="s">
         <v>2</v>
@@ -15222,13 +15271,13 @@
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
-        <v>171</v>
+        <v>178</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>100</v>
+        <v>107</v>
       </c>
       <c r="D35" s="11" t="s">
         <v>2</v>
@@ -15256,7 +15305,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>173</v>
+        <v>180</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -15278,13 +15327,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>174</v>
+        <v>181</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>175</v>
+        <v>182</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>2</v>
@@ -15292,13 +15341,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>177</v>
+        <v>184</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>178</v>
+        <v>185</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>2</v>
@@ -15306,27 +15355,27 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>179</v>
+        <v>186</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>180</v>
+        <v>187</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>181</v>
+        <v>188</v>
       </c>
       <c r="D5" s="11" t="s">
-        <v>182</v>
+        <v>189</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>183</v>
+        <v>190</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>184</v>
+        <v>191</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>185</v>
+        <v>192</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>2</v>
@@ -15334,13 +15383,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>186</v>
+        <v>193</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>187</v>
+        <v>194</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>188</v>
+        <v>195</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>2</v>
@@ -15348,13 +15397,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>189</v>
+        <v>196</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>190</v>
+        <v>197</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>2</v>
@@ -15362,13 +15411,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>192</v>
+        <v>199</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>193</v>
+        <v>200</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>194</v>
+        <v>201</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>2</v>
@@ -15376,13 +15425,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>195</v>
+        <v>202</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>196</v>
+        <v>203</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>197</v>
+        <v>204</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>2</v>
@@ -15390,13 +15439,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>198</v>
+        <v>205</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>199</v>
+        <v>206</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>2</v>
@@ -15404,13 +15453,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>201</v>
+        <v>208</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>202</v>
+        <v>209</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>203</v>
+        <v>210</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>2</v>
@@ -15418,13 +15467,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>204</v>
+        <v>211</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>205</v>
+        <v>212</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>206</v>
+        <v>213</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>2</v>
@@ -15432,13 +15481,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>207</v>
+        <v>214</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>208</v>
+        <v>215</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>209</v>
+        <v>216</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>2</v>
@@ -15446,13 +15495,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>210</v>
+        <v>217</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>211</v>
+        <v>218</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>212</v>
+        <v>219</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>2</v>
@@ -15460,13 +15509,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>213</v>
+        <v>220</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>214</v>
+        <v>221</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>215</v>
+        <v>222</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>2</v>
@@ -15474,13 +15523,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>216</v>
+        <v>223</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>217</v>
+        <v>224</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>218</v>
+        <v>225</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>2</v>
@@ -15488,27 +15537,27 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>219</v>
+        <v>226</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>220</v>
+        <v>227</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="D18" s="11" t="s">
-        <v>222</v>
+        <v>229</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>223</v>
+        <v>230</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>224</v>
+        <v>231</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>2</v>
@@ -15516,13 +15565,13 @@
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" s="8" t="s">
-        <v>225</v>
+        <v>232</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>226</v>
+        <v>233</v>
       </c>
       <c r="C20" s="10" t="s">
-        <v>227</v>
+        <v>234</v>
       </c>
       <c r="D20" s="11" t="s">
         <v>2</v>
@@ -15530,13 +15579,13 @@
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" s="8" t="s">
-        <v>228</v>
+        <v>235</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>229</v>
+        <v>236</v>
       </c>
       <c r="C21" s="10" t="s">
-        <v>230</v>
+        <v>237</v>
       </c>
       <c r="D21" s="11" t="s">
         <v>2</v>
@@ -15544,27 +15593,27 @@
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="8" t="s">
-        <v>231</v>
+        <v>238</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>232</v>
+        <v>239</v>
       </c>
       <c r="C22" s="10" t="s">
-        <v>233</v>
+        <v>240</v>
       </c>
       <c r="D22" s="11" t="s">
-        <v>234</v>
+        <v>241</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
-        <v>235</v>
+        <v>242</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>236</v>
+        <v>243</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>237</v>
+        <v>244</v>
       </c>
       <c r="D23" s="11" t="s">
         <v>2</v>
@@ -15572,13 +15621,13 @@
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
-        <v>238</v>
+        <v>245</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>239</v>
+        <v>246</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>240</v>
+        <v>247</v>
       </c>
       <c r="D24" s="11" t="s">
         <v>2</v>
@@ -15586,13 +15635,13 @@
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
-        <v>241</v>
+        <v>248</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>242</v>
+        <v>249</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>243</v>
+        <v>250</v>
       </c>
       <c r="D25" s="11" t="s">
         <v>2</v>
@@ -15600,13 +15649,13 @@
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="8" t="s">
-        <v>244</v>
+        <v>251</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>245</v>
+        <v>252</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>246</v>
+        <v>253</v>
       </c>
       <c r="D26" s="11" t="s">
         <v>2</v>
@@ -15614,13 +15663,13 @@
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="8" t="s">
-        <v>247</v>
+        <v>254</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>248</v>
+        <v>255</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>249</v>
+        <v>256</v>
       </c>
       <c r="D27" s="11" t="s">
         <v>2</v>
@@ -15628,27 +15677,27 @@
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
-        <v>250</v>
+        <v>257</v>
       </c>
       <c r="B28" s="9" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D28" s="11" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="8" t="s">
-        <v>253</v>
+        <v>260</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>254</v>
+        <v>261</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>255</v>
+        <v>262</v>
       </c>
       <c r="D29" s="11" t="s">
         <v>2</v>
@@ -15656,10 +15705,10 @@
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="8" t="s">
-        <v>256</v>
+        <v>263</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>257</v>
+        <v>264</v>
       </c>
       <c r="C30" s="10" t="s">
         <v>2</v>
@@ -15690,7 +15739,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>258</v>
+        <v>265</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -15712,27 +15761,27 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>259</v>
+        <v>266</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>260</v>
+        <v>267</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>261</v>
+        <v>268</v>
       </c>
       <c r="D3" s="11" t="s">
-        <v>262</v>
+        <v>269</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>263</v>
+        <v>270</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>264</v>
+        <v>271</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>265</v>
+        <v>272</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>2</v>
@@ -15740,13 +15789,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>266</v>
+        <v>273</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>267</v>
+        <v>274</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>268</v>
+        <v>275</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>2</v>
@@ -15754,10 +15803,10 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>269</v>
+        <v>276</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>270</v>
+        <v>277</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>2</v>
@@ -15768,13 +15817,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>271</v>
+        <v>278</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>272</v>
+        <v>279</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>2</v>
@@ -15782,41 +15831,41 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>274</v>
+        <v>281</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>275</v>
+        <v>282</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>276</v>
+        <v>283</v>
       </c>
       <c r="D8" s="11" t="s">
-        <v>277</v>
+        <v>284</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>278</v>
+        <v>285</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>279</v>
+        <v>286</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>280</v>
+        <v>287</v>
       </c>
       <c r="D9" s="11" t="s">
-        <v>281</v>
+        <v>288</v>
       </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>283</v>
+        <v>290</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>191</v>
+        <v>198</v>
       </c>
       <c r="D10" s="11" t="s">
         <v>2</v>
@@ -15824,13 +15873,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>284</v>
+        <v>291</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>285</v>
+        <v>292</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>286</v>
+        <v>293</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>2</v>
@@ -15838,13 +15887,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>287</v>
+        <v>294</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>288</v>
+        <v>295</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>176</v>
+        <v>183</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>2</v>
@@ -15852,13 +15901,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>2</v>
@@ -15866,13 +15915,13 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="B14" s="9" t="s">
-        <v>293</v>
+        <v>300</v>
       </c>
       <c r="C14" s="10" t="s">
-        <v>200</v>
+        <v>207</v>
       </c>
       <c r="D14" s="11" t="s">
         <v>2</v>
@@ -15880,13 +15929,13 @@
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
-        <v>294</v>
+        <v>301</v>
       </c>
       <c r="B15" s="9" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="C15" s="10" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="D15" s="11" t="s">
         <v>2</v>
@@ -15894,13 +15943,13 @@
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="C16" s="10" t="s">
-        <v>151</v>
+        <v>158</v>
       </c>
       <c r="D16" s="11" t="s">
         <v>2</v>
@@ -15908,13 +15957,13 @@
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
-        <v>299</v>
+        <v>306</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>300</v>
+        <v>307</v>
       </c>
       <c r="C17" s="10" t="s">
-        <v>301</v>
+        <v>308</v>
       </c>
       <c r="D17" s="11" t="s">
         <v>2</v>
@@ -15922,13 +15971,13 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="8" t="s">
-        <v>302</v>
+        <v>309</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>303</v>
+        <v>310</v>
       </c>
       <c r="C18" s="10" t="s">
-        <v>304</v>
+        <v>311</v>
       </c>
       <c r="D18" s="11" t="s">
         <v>2</v>
@@ -15936,13 +15985,13 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="8" t="s">
-        <v>305</v>
+        <v>312</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>306</v>
+        <v>313</v>
       </c>
       <c r="C19" s="10" t="s">
-        <v>307</v>
+        <v>314</v>
       </c>
       <c r="D19" s="11" t="s">
         <v>2</v>
@@ -15975,7 +16024,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -15997,13 +16046,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B3" s="9" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
       <c r="D3" s="11" t="s">
         <v>2</v>
@@ -16011,13 +16060,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="8" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B4" s="9" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
       <c r="D4" s="11" t="s">
         <v>2</v>
@@ -16025,13 +16074,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B5" s="9" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
       <c r="D5" s="11" t="s">
         <v>2</v>
@@ -16039,13 +16088,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="8" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B6" s="9" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
       <c r="D6" s="11" t="s">
         <v>2</v>
@@ -16053,13 +16102,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="8" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B7" s="9" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
       <c r="D7" s="11" t="s">
         <v>2</v>
@@ -16067,13 +16116,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" s="8" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B8" s="9" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
       <c r="D8" s="11" t="s">
         <v>2</v>
@@ -16081,13 +16130,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" s="8" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B9" s="9" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
       <c r="D9" s="11" t="s">
         <v>2</v>
@@ -16095,27 +16144,27 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="8" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="B10" s="9" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="C10" s="10" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="D10" s="11" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="8" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
       <c r="B11" s="9" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="C11" s="10" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="D11" s="11" t="s">
         <v>2</v>
@@ -16123,13 +16172,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="8" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="B12" s="9" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="C12" s="10" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="D12" s="11" t="s">
         <v>2</v>
@@ -16137,13 +16186,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="B13" s="9" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="C13" s="10" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="D13" s="11" t="s">
         <v>2</v>
@@ -16170,7 +16219,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -16184,57 +16233,57 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="G2" s="7" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
       <c r="H2" s="7" t="s">
-        <v>350</v>
+        <v>357</v>
       </c>
       <c r="I2" s="7" t="s">
-        <v>351</v>
+        <v>358</v>
       </c>
       <c r="J2" s="7" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
+        <v>360</v>
+      </c>
+      <c r="C3" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="D3" s="10" t="s">
         <v>353</v>
       </c>
-      <c r="C3" s="10" t="s">
+      <c r="E3" s="10" t="s">
         <v>354</v>
       </c>
-      <c r="D3" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>347</v>
-      </c>
       <c r="F3" s="10" t="s">
         <v>2</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="H3" s="10" t="s">
         <v>2</v>
@@ -16243,25 +16292,25 @@
         <v>2</v>
       </c>
       <c r="J3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>356</v>
+        <v>363</v>
       </c>
       <c r="C4" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="E4" s="10" t="s">
         <v>354</v>
       </c>
-      <c r="D4" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="E4" s="10" t="s">
-        <v>347</v>
-      </c>
       <c r="F4" s="10" t="s">
         <v>2</v>
       </c>
@@ -16275,30 +16324,30 @@
         <v>2</v>
       </c>
       <c r="J4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>357</v>
+        <v>364</v>
       </c>
       <c r="C5" s="10" t="s">
+        <v>361</v>
+      </c>
+      <c r="D5" s="10" t="s">
+        <v>353</v>
+      </c>
+      <c r="E5" s="10" t="s">
         <v>354</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>346</v>
-      </c>
-      <c r="E5" s="10" t="s">
-        <v>347</v>
-      </c>
       <c r="F5" s="10" t="s">
         <v>2</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>355</v>
+        <v>362</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>2</v>
@@ -16307,7 +16356,7 @@
         <v>2</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
@@ -18274,7 +18323,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>358</v>
+        <v>365</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -18285,39 +18334,39 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="D2" s="7" t="s">
+        <v>366</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>357</v>
+      </c>
+      <c r="F2" s="7" t="s">
+        <v>367</v>
+      </c>
+      <c r="G2" s="7" t="s">
         <v>359</v>
-      </c>
-      <c r="E2" s="7" t="s">
-        <v>350</v>
-      </c>
-      <c r="F2" s="7" t="s">
-        <v>360</v>
-      </c>
-      <c r="G2" s="7" t="s">
-        <v>352</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="C3" s="10" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>2</v>
@@ -18326,21 +18375,21 @@
         <v>2</v>
       </c>
       <c r="G3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>2</v>
@@ -18349,21 +18398,21 @@
         <v>2</v>
       </c>
       <c r="G4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>2</v>
@@ -18372,21 +18421,21 @@
         <v>2</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>361</v>
+        <v>368</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>362</v>
+        <v>369</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>363</v>
+        <v>370</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>2</v>
@@ -18395,7 +18444,7 @@
         <v>2</v>
       </c>
       <c r="G6" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.25">
@@ -19813,7 +19862,7 @@
   <sheetData>
     <row r="1" ht="30" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>364</v>
+        <v>371</v>
       </c>
       <c r="B1" s="6"/>
       <c r="C1" s="6"/>
@@ -19823,182 +19872,182 @@
     </row>
     <row r="2" ht="22" customHeight="1" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A2" s="7" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
       <c r="B2" s="7" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
       <c r="C2" s="7" t="s">
-        <v>365</v>
+        <v>372</v>
       </c>
       <c r="D2" s="7" t="s">
-        <v>366</v>
+        <v>373</v>
       </c>
       <c r="E2" s="7" t="s">
-        <v>367</v>
+        <v>374</v>
       </c>
       <c r="F2" s="7" t="s">
-        <v>352</v>
+        <v>359</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B3" s="10" t="s">
-        <v>368</v>
+        <v>375</v>
       </c>
       <c r="C3" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D3" s="10" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E3" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F3" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>370</v>
+        <v>377</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E4" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F4" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B5" s="10" t="s">
-        <v>371</v>
+        <v>378</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E5" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F5" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B6" s="10" t="s">
-        <v>372</v>
+        <v>379</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E6" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F6" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B7" s="10" t="s">
-        <v>373</v>
+        <v>380</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E7" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F7" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B8" s="10" t="s">
-        <v>374</v>
+        <v>381</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E8" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F8" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>375</v>
+        <v>382</v>
       </c>
       <c r="C9" s="10" t="s">
         <v>2</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>369</v>
+        <v>376</v>
       </c>
       <c r="E9" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F9" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
       <c r="B10" s="10" t="s">
+        <v>383</v>
+      </c>
+      <c r="C10" s="10" t="s">
+        <v>2</v>
+      </c>
+      <c r="D10" s="10" t="s">
         <v>376</v>
       </c>
-      <c r="C10" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="D10" s="10" t="s">
-        <v>369</v>
-      </c>
       <c r="E10" s="10" t="s">
         <v>2</v>
       </c>
       <c r="F10" s="10" t="s">
-        <v>273</v>
+        <v>280</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">

</xml_diff>